<commit_message>
Recalibrate bear and bull around the v3 base
Bear is now a hard deceleration, not a collapse: OpenAI $150B and
Anthropic $200B in 2030 (exit run-rates $58B -> $159B and $100B -> $211B,
growth slowing to ~10% by 2030; 15-16 GW average; yield $20-24B per
inference GW). Bull is the stated capacity path without haircut at flat
yield, ~1.4x base: OpenAI $484B, Anthropic $584B. Base unchanged (= v3).
Demand, supply and momentum lenses agree within ~3% in every scenario.
Sensitivity grids and the doc updated; 894 formulas, zero errors,
verified against Python and v3.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019aUdnej14hr8ouHNhrtwo4
</commit_message>
<xml_diff>
--- a/ai_labs_2030/model/AI_labs_revenue_2030_bottomup.xlsx
+++ b/ai_labs_2030/model/AI_labs_revenue_2030_bottomup.xlsx
@@ -325,7 +325,7 @@
     <t xml:space="preserve">AI spend / salary - developers</t>
   </si>
   <si>
-    <t xml:space="preserve">Base $12.6k/dev/yr is what the v3 revenue needs; 2026: Claude Code enterprise avg $150-250/mo = $1.8-3k/yr; heavy agent users &gt;$1k/mo</t>
+    <t xml:space="preserve">Base $12.6k/dev/yr is what the v3 revenue needs; bear $7.9k, bull $14.8k; 2026: Claude Code enterprise avg $150-250/mo = $1.8-3k/yr; heavy agent users &gt;$1k/mo</t>
   </si>
   <si>
     <t xml:space="preserve">ratio_pro</t>
@@ -577,7 +577,7 @@
     <t xml:space="preserve">GW</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 OpenAI_breakeven_model_MBI_vBTG_v3.xlsx Model!I29 (year-end 22.1 GW after the 26.4% budget haircut on the 30 GW path); bull = full stated path avg(25,30)</t>
+    <t xml:space="preserve">Base = v3 OpenAI_breakeven_model_MBI_vBTG_v3.xlsx Model!I29 (year-end 22.1 GW after the 26.4% budget haircut on the 30 GW path); bear 15 GW (build slows); bull = full stated path avg(25,30)</t>
   </si>
   <si>
     <t xml:space="preserve">oai_inf_share_avg</t>
@@ -595,7 +595,7 @@
     <t xml:space="preserve">OpenAI revenue per average inference GW-year 2030 ($B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 OpenAI_breakeven_model_MBI_vBTG_v3.xlsx Model!I101 (breakeven yield); 2026E $27.1B (E101); exit-ARR yield 2026E $32.9B</t>
+    <t xml:space="preserve">Base = v3 OpenAI_breakeven_model_MBI_vBTG_v3.xlsx Model!I101 (breakeven yield); bear $20B (price deflation outruns volume); bull $30B (deck); 2026E $27.1B (E101)</t>
   </si>
   <si>
     <t xml:space="preserve">oai_cost_inf_gw</t>
@@ -643,7 +643,7 @@
     <t xml:space="preserve">Anthropic revenue per average inference GW-year 2030 ($B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 Anthropic_model_MBI_vBTG_v3.xlsx Model!I88: 2026E $40.2B then -6%/yr 2027-29 and -5.3% in 2030; v3 breakeven yield memo $30.1B (I94)</t>
+    <t xml:space="preserve">Base = v3 Anthropic_model_MBI_vBTG_v3.xlsx Model!I88: 2026E $40.2B then -6%/yr 2027-29 and -5.3% in 2030; bear $24B (-12%/yr); bull $40B (flat at 2026E); v3 breakeven yield memo $30.1B (I94)</t>
   </si>
   <si>
     <t xml:space="preserve">ant_cost_inf_gw</t>
@@ -727,7 +727,7 @@
     <t xml:space="preserve">OpenAI exit-2026 run-rate ($B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 OpenAI_breakeven_model_MBI_vBTG_v3.xlsx Model!E105; &gt;$40B run-rate Aug-26 (+35% QTD)</t>
+    <t xml:space="preserve">Base = v3 OpenAI_breakeven_model_MBI_vBTG_v3.xlsx Model!E105; &gt;$40B run-rate Aug-26 (+35% QTD); bear $58B</t>
   </si>
   <si>
     <t xml:space="preserve">ant_rr26</t>
@@ -736,7 +736,7 @@
     <t xml:space="preserve">Anthropic exit-2026 run-rate ($B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 Anthropic_model_MBI_vBTG_v3.xlsx Model!E90; $65B run-rate end-Jul-26</t>
+    <t xml:space="preserve">Base = v3 Anthropic_model_MBI_vBTG_v3.xlsx Model!E90; $65B run-rate end-Jul-26; bear keeps $100B</t>
   </si>
   <si>
     <t xml:space="preserve">oai_g27</t>
@@ -745,7 +745,7 @@
     <t xml:space="preserve">OpenAI exit run-rate growth 2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 exit ARR path (Model!E105:I105)</t>
+    <t xml:space="preserve">Base = v3 exit ARR path (Model!E105:I105); bear: growth decelerates to ~10% by 2030 (calendar 2030 ~$150B); bull ~$470B</t>
   </si>
   <si>
     <t xml:space="preserve">oai_g28</t>
@@ -772,7 +772,7 @@
     <t xml:space="preserve">Anthropic exit run-rate growth 2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Base = v3 exit ARR path (Model!E90:I90)</t>
+    <t xml:space="preserve">Base = v3 exit ARR path (Model!E90:I90); bear: ~8% by 2030 (calendar 2030 ~$200B); bull ~$570B</t>
   </si>
   <si>
     <t xml:space="preserve">ant_g28</t>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">OpenAI!C27</f>
-        <v>91.82922</v>
+        <v>149.953848</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">OpenAI!D27</f>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D5" s="5" t="n">
         <f aca="false">OpenAI!E27</f>
-        <v>765.0088</v>
+        <v>483.83538</v>
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">OpenAI!F27</f>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">OpenAI!C38</f>
-        <v>147.84</v>
+        <v>150</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">OpenAI!D38</f>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">OpenAI!E38</f>
-        <v>660</v>
+        <v>478.5</v>
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">OpenAI!F38</f>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">OpenAI!C56</f>
-        <v>119.886</v>
+        <v>151.772544</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">OpenAI!D56</f>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">OpenAI!E56</f>
-        <v>455.2275</v>
+        <v>472.03416</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">OpenAI!F56</f>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">OpenAI!C41</f>
-        <v>13.6650625</v>
+        <v>19.9938464</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">OpenAI!D41</f>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D8" s="6" t="n">
         <f aca="false">OpenAI!E41</f>
-        <v>46.3641696969697</v>
+        <v>30.3345065830721</v>
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">OpenAI!F41</f>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">Anthropic!C27</f>
-        <v>101.37187</v>
+        <v>199.61578</v>
       </c>
       <c r="C9" s="5" t="n">
         <f aca="false">Anthropic!D27</f>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">Anthropic!E27</f>
-        <v>779.8784</v>
+        <v>584.47366</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">Anthropic!F27</f>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Anthropic!C38</f>
-        <v>180</v>
+        <v>199.68</v>
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Anthropic!D38</f>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">Anthropic!E38</f>
-        <v>675</v>
+        <v>580</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">Anthropic!F38</f>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Anthropic!C56</f>
-        <v>167.479648</v>
+        <v>202.879872</v>
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">Anthropic!D56</f>
@@ -2804,7 +2804,7 @@
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">Anthropic!E56</f>
-        <v>568.8144</v>
+        <v>567.61056</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">Anthropic!F56</f>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">Anthropic!C41</f>
-        <v>14.0794263888889</v>
+        <v>23.99228125</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">Anthropic!D41</f>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="D12" s="6" t="n">
         <f aca="false">Anthropic!E41</f>
-        <v>51.9918933333333</v>
+        <v>40.3085282758621</v>
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">Anthropic!F41</f>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">B5+B9</f>
-        <v>193.20109</v>
+        <v>349.569628</v>
       </c>
       <c r="C13" s="8" t="n">
         <f aca="false">C5+C9</f>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="D13" s="8" t="n">
         <f aca="false">D5+D9</f>
-        <v>1544.8872</v>
+        <v>1068.30904</v>
       </c>
       <c r="E13" s="8" t="n">
         <f aca="false">E5+E9</f>
@@ -3438,13 +3438,13 @@
         <v>67</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>42</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G6" s="17" t="n">
         <v>42</v>
@@ -3464,13 +3464,13 @@
         <v>67</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E7" s="15" t="n">
         <v>220</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="G7" s="17" t="n">
         <v>220</v>
@@ -3490,13 +3490,13 @@
         <v>67</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="E8" s="15" t="n">
         <v>790</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>815</v>
+        <v>800</v>
       </c>
       <c r="G8" s="17" t="n">
         <v>790</v>
@@ -3522,7 +3522,7 @@
         <v>75</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G9" s="17" t="n">
         <v>75</v>
@@ -3548,7 +3548,7 @@
         <v>60</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G10" s="17" t="n">
         <v>60</v>
@@ -3574,7 +3574,7 @@
         <v>30</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G11" s="17" t="n">
         <v>30</v>
@@ -3606,13 +3606,13 @@
         <v>88</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0.7</v>
+        <v>0.78</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>0.85</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="G13" s="19" t="n">
         <v>0.85</v>
@@ -3632,13 +3632,13 @@
         <v>88</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>0.35</v>
+        <v>0.42</v>
       </c>
       <c r="E14" s="18" t="n">
         <v>0.5</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="G14" s="19" t="n">
         <v>0.5</v>
@@ -3658,13 +3658,13 @@
         <v>88</v>
       </c>
       <c r="D15" s="18" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="E15" s="18" t="n">
         <v>0.3</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.4</v>
+        <v>0.36</v>
       </c>
       <c r="G15" s="19" t="n">
         <v>0.3</v>
@@ -3696,13 +3696,13 @@
         <v>88</v>
       </c>
       <c r="D17" s="18" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
       <c r="E17" s="18" t="n">
         <v>0.168</v>
       </c>
       <c r="F17" s="18" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="G17" s="19" t="n">
         <v>0.168</v>
@@ -3722,13 +3722,13 @@
         <v>88</v>
       </c>
       <c r="D18" s="18" t="n">
-        <v>0.02</v>
+        <v>0.026</v>
       </c>
       <c r="E18" s="18" t="n">
         <v>0.045</v>
       </c>
       <c r="F18" s="18" t="n">
-        <v>0.06</v>
+        <v>0.052</v>
       </c>
       <c r="G18" s="19" t="n">
         <v>0.045</v>
@@ -3748,13 +3748,13 @@
         <v>88</v>
       </c>
       <c r="D19" s="18" t="n">
-        <v>0.008</v>
+        <v>0.009</v>
       </c>
       <c r="E19" s="18" t="n">
         <v>0.014</v>
       </c>
       <c r="F19" s="18" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
       <c r="G19" s="19" t="n">
         <v>0.014</v>
@@ -3786,13 +3786,13 @@
         <v>88</v>
       </c>
       <c r="D21" s="18" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="E21" s="18" t="n">
         <v>0.455737850695834</v>
       </c>
       <c r="F21" s="18" t="n">
-        <v>0.48</v>
+        <v>0.46</v>
       </c>
       <c r="G21" s="19" t="n">
         <v>0.455737850695834</v>
@@ -3812,13 +3812,13 @@
         <v>88</v>
       </c>
       <c r="D22" s="18" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="E22" s="18" t="n">
         <v>0.173402694411098</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="G22" s="19" t="n">
         <v>0.173402694411098</v>
@@ -3838,13 +3838,13 @@
         <v>88</v>
       </c>
       <c r="D23" s="18" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="E23" s="18" t="n">
         <v>0.185185185185185</v>
       </c>
       <c r="F23" s="18" t="n">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="G23" s="19" t="n">
         <v>0.185185185185185</v>
@@ -3864,13 +3864,13 @@
         <v>88</v>
       </c>
       <c r="D24" s="18" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="E24" s="18" t="n">
         <v>0.228956228956229</v>
       </c>
       <c r="F24" s="18" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="G24" s="19" t="n">
         <v>0.228956228956229</v>
@@ -3890,13 +3890,13 @@
         <v>88</v>
       </c>
       <c r="D25" s="18" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E25" s="18" t="n">
         <v>0.0803697006228652</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="G25" s="19" t="n">
         <v>0.0803697006228652</v>
@@ -3916,13 +3916,13 @@
         <v>88</v>
       </c>
       <c r="D26" s="18" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="E26" s="18" t="n">
         <v>0.180831826401447</v>
       </c>
       <c r="F26" s="18" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="G26" s="19" t="n">
         <v>0.180831826401447</v>
@@ -3960,7 +3960,7 @@
         <v>8</v>
       </c>
       <c r="F28" s="20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G28" s="21" t="n">
         <v>8</v>
@@ -3980,13 +3980,13 @@
         <v>88</v>
       </c>
       <c r="D29" s="18" t="n">
-        <v>0.07</v>
+        <v>0.09</v>
       </c>
       <c r="E29" s="18" t="n">
         <v>0.125</v>
       </c>
       <c r="F29" s="18" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="G29" s="19" t="n">
         <v>0.125</v>
@@ -4006,13 +4006,13 @@
         <v>88</v>
       </c>
       <c r="D30" s="18" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="E30" s="18" t="n">
         <v>0.3</v>
       </c>
       <c r="F30" s="18" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="G30" s="19" t="n">
         <v>0.3</v>
@@ -4032,14 +4032,14 @@
         <v>88</v>
       </c>
       <c r="D31" s="18" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E31" s="22" t="n">
         <f aca="false">IF(Anthropic!$D$15=0,0,(Inputs!$E$94-(Anthropic!$D$19+Anthropic!$D$20+Anthropic!$D$21+Anthropic!$D$23+Anthropic!$D$24+Anthropic!$D$25+Anthropic!$D$26))/Anthropic!$D$15)</f>
         <v>0.43739334954074</v>
       </c>
       <c r="F31" s="18" t="n">
-        <v>0.45</v>
+        <v>0.43</v>
       </c>
       <c r="G31" s="19" t="n">
         <v>0.43739334954074</v>
@@ -4059,14 +4059,14 @@
         <v>88</v>
       </c>
       <c r="D32" s="18" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E32" s="22" t="n">
         <f aca="false">IF(OpenAI!$D$15=0,0,(Inputs!$E$78-(OpenAI!$D$19+OpenAI!$D$20+OpenAI!$D$21+OpenAI!$D$23+OpenAI!$D$24+OpenAI!$D$25+OpenAI!$D$26))/OpenAI!$D$15)</f>
         <v>0.157728647478893</v>
       </c>
       <c r="F32" s="18" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="G32" s="19" t="n">
         <v>0.157728647478893</v>
@@ -4098,13 +4098,13 @@
         <v>67</v>
       </c>
       <c r="D34" s="15" t="n">
-        <v>1500</v>
+        <v>1600</v>
       </c>
       <c r="E34" s="15" t="n">
         <v>2000</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>2500</v>
+        <v>2300</v>
       </c>
       <c r="G34" s="17" t="n">
         <v>2000</v>
@@ -4124,13 +4124,13 @@
         <v>88</v>
       </c>
       <c r="D35" s="18" t="n">
-        <v>0.045</v>
+        <v>0.052</v>
       </c>
       <c r="E35" s="18" t="n">
         <v>0.065</v>
       </c>
       <c r="F35" s="18" t="n">
-        <v>0.09</v>
+        <v>0.075</v>
       </c>
       <c r="G35" s="19" t="n">
         <v>0.065</v>
@@ -4150,13 +4150,13 @@
         <v>151</v>
       </c>
       <c r="D36" s="23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E36" s="23" t="n">
         <v>20.5</v>
       </c>
       <c r="F36" s="23" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G36" s="24" t="n">
         <v>20.5</v>
@@ -4176,13 +4176,13 @@
         <v>155</v>
       </c>
       <c r="D37" s="25" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E37" s="25" t="n">
         <v>40</v>
       </c>
       <c r="F37" s="25" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="G37" s="26" t="n">
         <v>40</v>
@@ -4202,13 +4202,13 @@
         <v>159</v>
       </c>
       <c r="D38" s="27" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="E38" s="27" t="n">
         <v>480</v>
       </c>
       <c r="F38" s="27" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="G38" s="28" t="n">
         <v>480</v>
@@ -4234,7 +4234,7 @@
         <v>0.025</v>
       </c>
       <c r="F39" s="18" t="n">
-        <v>0.03</v>
+        <v>0.027</v>
       </c>
       <c r="G39" s="19" t="n">
         <v>0.025</v>
@@ -4266,13 +4266,13 @@
         <v>67</v>
       </c>
       <c r="D41" s="15" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="E41" s="15" t="n">
         <v>250</v>
       </c>
       <c r="F41" s="15" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="G41" s="17" t="n">
         <v>250</v>
@@ -4292,13 +4292,13 @@
         <v>88</v>
       </c>
       <c r="D42" s="18" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="E42" s="18" t="n">
         <v>0.12</v>
       </c>
       <c r="F42" s="18" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="G42" s="19" t="n">
         <v>0.12</v>
@@ -4318,13 +4318,13 @@
         <v>151</v>
       </c>
       <c r="D43" s="23" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E43" s="23" t="n">
         <v>40</v>
       </c>
       <c r="F43" s="23" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G43" s="24" t="n">
         <v>40</v>
@@ -4356,13 +4356,13 @@
         <v>159</v>
       </c>
       <c r="D45" s="27" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E45" s="27" t="n">
         <v>8</v>
       </c>
       <c r="F45" s="27" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G45" s="28" t="n">
         <v>8</v>
@@ -4382,13 +4382,13 @@
         <v>159</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E46" s="27" t="n">
         <v>12</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G46" s="28" t="n">
         <v>12</v>
@@ -4420,7 +4420,7 @@
         <v>182</v>
       </c>
       <c r="D48" s="29" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E48" s="29" t="n">
         <v>20.2379725666731</v>
@@ -4446,13 +4446,13 @@
         <v>88</v>
       </c>
       <c r="D49" s="18" t="n">
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="E49" s="18" t="n">
         <v>0.540909090909088</v>
       </c>
       <c r="F49" s="18" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="G49" s="19" t="n">
         <v>0.540909090909088</v>
@@ -4472,13 +4472,13 @@
         <v>159</v>
       </c>
       <c r="D50" s="27" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E50" s="27" t="n">
         <v>30.8853183090816</v>
       </c>
       <c r="F50" s="27" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="G50" s="28" t="n">
         <v>30.8853183090816</v>
@@ -4498,13 +4498,13 @@
         <v>159</v>
       </c>
       <c r="D51" s="27" t="n">
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="E51" s="27" t="n">
         <v>11.7004035197334</v>
       </c>
       <c r="F51" s="27" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="G51" s="28" t="n">
         <v>11.7004035197334</v>
@@ -4562,7 +4562,7 @@
         <v>182</v>
       </c>
       <c r="D54" s="29" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E54" s="29" t="n">
         <v>22.5</v>
@@ -4588,13 +4588,13 @@
         <v>88</v>
       </c>
       <c r="D55" s="18" t="n">
-        <v>0.48</v>
+        <v>0.52</v>
       </c>
       <c r="E55" s="18" t="n">
         <v>0.541111111111111</v>
       </c>
       <c r="F55" s="18" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="G55" s="19" t="n">
         <v>0.541111111111111</v>
@@ -4614,13 +4614,13 @@
         <v>159</v>
       </c>
       <c r="D56" s="27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E56" s="27" t="n">
         <v>34.9583576888889</v>
       </c>
       <c r="F56" s="27" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G56" s="28" t="n">
         <v>34.9583576888889</v>
@@ -4640,13 +4640,13 @@
         <v>159</v>
       </c>
       <c r="D57" s="27" t="n">
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="E57" s="27" t="n">
         <v>12</v>
       </c>
       <c r="F57" s="27" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="G57" s="28" t="n">
         <v>12</v>
@@ -4858,7 +4858,7 @@
         <v>159</v>
       </c>
       <c r="D67" s="27" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E67" s="27" t="n">
         <v>60</v>
@@ -4884,7 +4884,7 @@
         <v>159</v>
       </c>
       <c r="D68" s="27" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E68" s="27" t="n">
         <v>100</v>
@@ -4910,13 +4910,13 @@
         <v>88</v>
       </c>
       <c r="D69" s="18" t="n">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="E69" s="18" t="n">
         <v>1.27409281012993</v>
       </c>
       <c r="F69" s="18" t="n">
-        <v>1.4</v>
+        <v>1.35</v>
       </c>
       <c r="G69" s="19" t="n">
         <v>1.27409281012993</v>
@@ -4936,13 +4936,13 @@
         <v>88</v>
       </c>
       <c r="D70" s="18" t="n">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="E70" s="18" t="n">
         <v>0.657971176976747</v>
       </c>
       <c r="F70" s="18" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="G70" s="19" t="n">
         <v>0.657971176976747</v>
@@ -4960,13 +4960,13 @@
         <v>88</v>
       </c>
       <c r="D71" s="18" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="E71" s="18" t="n">
         <v>0.342290767401188</v>
       </c>
       <c r="F71" s="18" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="G71" s="19" t="n">
         <v>0.342290767401188</v>
@@ -4984,13 +4984,13 @@
         <v>88</v>
       </c>
       <c r="D72" s="18" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="E72" s="18" t="n">
         <v>0.226846830456758</v>
       </c>
       <c r="F72" s="18" t="n">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="G72" s="19" t="n">
         <v>0.226846830456758</v>
@@ -5008,13 +5008,13 @@
         <v>88</v>
       </c>
       <c r="D73" s="18" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="E73" s="18" t="n">
         <v>0.94533333333333</v>
       </c>
       <c r="F73" s="18" t="n">
-        <v>1.1</v>
+        <v>1.05</v>
       </c>
       <c r="G73" s="19" t="n">
         <v>0.94533333333333</v>
@@ -5034,7 +5034,7 @@
         <v>88</v>
       </c>
       <c r="D74" s="18" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="E74" s="18" t="n">
         <v>0.513324194653875</v>
@@ -5058,13 +5058,13 @@
         <v>88</v>
       </c>
       <c r="D75" s="18" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E75" s="18" t="n">
         <v>0.288431448922223</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="G75" s="19" t="n">
         <v>0.288431448922223</v>
@@ -5082,7 +5082,7 @@
         <v>88</v>
       </c>
       <c r="D76" s="18" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="E76" s="18" t="n">
         <v>0.244205727356943</v>
@@ -6018,7 +6018,7 @@
       </c>
       <c r="C6" s="31" t="n">
         <f aca="false">Inputs!$D$9*Inputs!$D$17*1000</f>
-        <v>5760</v>
+        <v>7920</v>
       </c>
       <c r="D6" s="31" t="n">
         <f aca="false">Inputs!$E$9*Inputs!$E$17*1000</f>
@@ -6026,7 +6026,7 @@
       </c>
       <c r="E6" s="31" t="n">
         <f aca="false">Inputs!$F$9*Inputs!$F$17*1000</f>
-        <v>16000</v>
+        <v>14820</v>
       </c>
       <c r="F6" s="31" t="n">
         <f aca="false">Inputs!$G$9*Inputs!$G$17*1000</f>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="C7" s="31" t="n">
         <f aca="false">Inputs!$D$10*Inputs!$D$18*1000</f>
-        <v>1140</v>
+        <v>1482</v>
       </c>
       <c r="D7" s="31" t="n">
         <f aca="false">Inputs!$E$10*Inputs!$E$18*1000</f>
@@ -6053,7 +6053,7 @@
       </c>
       <c r="E7" s="31" t="n">
         <f aca="false">Inputs!$F$10*Inputs!$F$18*1000</f>
-        <v>3900</v>
+        <v>3276</v>
       </c>
       <c r="F7" s="31" t="n">
         <f aca="false">Inputs!$G$10*Inputs!$G$18*1000</f>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="C8" s="31" t="n">
         <f aca="false">Inputs!$D$11*Inputs!$D$19*1000</f>
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="D8" s="31" t="n">
         <f aca="false">Inputs!$E$11*Inputs!$E$19*1000</f>
@@ -6078,7 +6078,7 @@
       </c>
       <c r="E8" s="31" t="n">
         <f aca="false">Inputs!$F$11*Inputs!$F$19*1000</f>
-        <v>640</v>
+        <v>527</v>
       </c>
       <c r="F8" s="31" t="n">
         <f aca="false">Inputs!$G$11*Inputs!$G$19*1000</f>
@@ -6095,7 +6095,7 @@
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">Inputs!$D$6*Inputs!$D$13</f>
-        <v>25.2</v>
+        <v>29.64</v>
       </c>
       <c r="D9" s="32" t="n">
         <f aca="false">Inputs!$E$6*Inputs!$E$13</f>
@@ -6103,7 +6103,7 @@
       </c>
       <c r="E9" s="32" t="n">
         <f aca="false">Inputs!$F$6*Inputs!$F$13</f>
-        <v>42.32</v>
+        <v>39.6</v>
       </c>
       <c r="F9" s="32" t="n">
         <f aca="false">Inputs!$G$6*Inputs!$G$13</f>
@@ -6122,7 +6122,7 @@
       </c>
       <c r="C10" s="32" t="n">
         <f aca="false">Inputs!$D$7*Inputs!$D$14</f>
-        <v>71.75</v>
+        <v>88.2</v>
       </c>
       <c r="D10" s="32" t="n">
         <f aca="false">Inputs!$E$7*Inputs!$E$14</f>
@@ -6130,7 +6130,7 @@
       </c>
       <c r="E10" s="32" t="n">
         <f aca="false">Inputs!$F$7*Inputs!$F$14</f>
-        <v>144</v>
+        <v>126.5</v>
       </c>
       <c r="F10" s="32" t="n">
         <f aca="false">Inputs!$G$7*Inputs!$G$14</f>
@@ -6147,7 +6147,7 @@
       </c>
       <c r="C11" s="32" t="n">
         <f aca="false">Inputs!$D$8*Inputs!$D$15</f>
-        <v>115.5</v>
+        <v>155</v>
       </c>
       <c r="D11" s="32" t="n">
         <f aca="false">Inputs!$E$8*Inputs!$E$15</f>
@@ -6155,7 +6155,7 @@
       </c>
       <c r="E11" s="32" t="n">
         <f aca="false">Inputs!$F$8*Inputs!$F$15</f>
-        <v>326</v>
+        <v>288</v>
       </c>
       <c r="F11" s="32" t="n">
         <f aca="false">Inputs!$G$8*Inputs!$G$15</f>
@@ -6172,7 +6172,7 @@
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">C9*C6/1000</f>
-        <v>145.152</v>
+        <v>234.7488</v>
       </c>
       <c r="D12" s="33" t="n">
         <f aca="false">D9*D6/1000</f>
@@ -6180,7 +6180,7 @@
       </c>
       <c r="E12" s="33" t="n">
         <f aca="false">E9*E6/1000</f>
-        <v>677.12</v>
+        <v>586.872</v>
       </c>
       <c r="F12" s="33" t="n">
         <f aca="false">F9*F6/1000</f>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="C13" s="33" t="n">
         <f aca="false">C10*C7/1000</f>
-        <v>81.795</v>
+        <v>130.7124</v>
       </c>
       <c r="D13" s="33" t="n">
         <f aca="false">D10*D7/1000</f>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="E13" s="33" t="n">
         <f aca="false">E10*E7/1000</f>
-        <v>561.6</v>
+        <v>414.414</v>
       </c>
       <c r="F13" s="33" t="n">
         <f aca="false">F10*F7/1000</f>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="C14" s="33" t="n">
         <f aca="false">C11*C8/1000</f>
-        <v>26.796</v>
+        <v>40.455</v>
       </c>
       <c r="D14" s="33" t="n">
         <f aca="false">D11*D8/1000</f>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="E14" s="33" t="n">
         <f aca="false">E11*E8/1000</f>
-        <v>208.64</v>
+        <v>151.776</v>
       </c>
       <c r="F14" s="33" t="n">
         <f aca="false">F11*F8/1000</f>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">Inputs!$D$28*Inputs!$D$29*Inputs!$D$30*1000</f>
-        <v>98</v>
+        <v>151.2</v>
       </c>
       <c r="D15" s="6" t="n">
         <f aca="false">Inputs!$E$28*Inputs!$E$29*Inputs!$E$30*1000</f>
@@ -6257,7 +6257,7 @@
       </c>
       <c r="E15" s="6" t="n">
         <f aca="false">Inputs!$F$28*Inputs!$F$29*Inputs!$F$30*1000</f>
-        <v>544</v>
+        <v>403.2</v>
       </c>
       <c r="F15" s="6" t="n">
         <f aca="false">Inputs!$G$28*Inputs!$G$29*Inputs!$G$30*1000</f>
@@ -6276,7 +6276,7 @@
       </c>
       <c r="C16" s="34" t="n">
         <f aca="false">SUM(C12:C15)</f>
-        <v>351.743</v>
+        <v>557.1162</v>
       </c>
       <c r="D16" s="34" t="n">
         <f aca="false">SUM(D12:D15)</f>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="E16" s="34" t="n">
         <f aca="false">SUM(E12:E15)</f>
-        <v>1991.36</v>
+        <v>1556.262</v>
       </c>
       <c r="F16" s="34" t="n">
         <f aca="false">SUM(F12:F15)</f>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="C19" s="6" t="n">
         <f aca="false">C12*Inputs!$D$22</f>
-        <v>20.32128</v>
+        <v>35.21232</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">D12*Inputs!$E$22</f>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">E12*Inputs!$F$22</f>
-        <v>162.5088</v>
+        <v>111.50568</v>
       </c>
       <c r="F19" s="6" t="n">
         <f aca="false">F12*Inputs!$G$22</f>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="C20" s="6" t="n">
         <f aca="false">C13*Inputs!$D$24</f>
-        <v>16.359</v>
+        <v>28.756728</v>
       </c>
       <c r="D20" s="6" t="n">
         <f aca="false">D13*Inputs!$E$24</f>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="E20" s="6" t="n">
         <f aca="false">E13*Inputs!$F$24</f>
-        <v>168.48</v>
+        <v>103.6035</v>
       </c>
       <c r="F20" s="6" t="n">
         <f aca="false">F13*Inputs!$G$24</f>
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C21" s="6" t="n">
         <f aca="false">C14*Inputs!$D$26</f>
-        <v>3.75144</v>
+        <v>6.4728</v>
       </c>
       <c r="D21" s="6" t="n">
         <f aca="false">D14*Inputs!$E$26</f>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">E14*Inputs!$F$26</f>
-        <v>52.16</v>
+        <v>30.3552</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">F14*Inputs!$G$26</f>
@@ -6389,7 +6389,7 @@
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">C15*Inputs!$D$32</f>
-        <v>11.76</v>
+        <v>21.168</v>
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">D15*Inputs!$E$32</f>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="E22" s="6" t="n">
         <f aca="false">E15*Inputs!$F$32</f>
-        <v>130.56</v>
+        <v>72.576</v>
       </c>
       <c r="F22" s="6" t="n">
         <f aca="false">F15*Inputs!$G$32</f>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">Inputs!$D$34*Inputs!$D$35*Inputs!$D$36*12/1000</f>
-        <v>12.15</v>
+        <v>15.9744</v>
       </c>
       <c r="D23" s="6" t="n">
         <f aca="false">Inputs!$E$34*Inputs!$E$35*Inputs!$E$36*12/1000</f>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="E23" s="6" t="n">
         <f aca="false">Inputs!$F$34*Inputs!$F$35*Inputs!$F$36*12/1000</f>
-        <v>64.8</v>
+        <v>45.54</v>
       </c>
       <c r="F23" s="6" t="n">
         <f aca="false">Inputs!$G$34*Inputs!$G$35*Inputs!$G$36*12/1000</f>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="C24" s="6" t="n">
         <f aca="false">Inputs!$D$34*(1-Inputs!$D$35)*Inputs!$D$37/1000</f>
-        <v>21.4875</v>
+        <v>33.3696</v>
       </c>
       <c r="D24" s="6" t="n">
         <f aca="false">Inputs!$E$34*(1-Inputs!$E$35)*Inputs!$E$37/1000</f>
@@ -6451,7 +6451,7 @@
       </c>
       <c r="E24" s="6" t="n">
         <f aca="false">Inputs!$F$34*(1-Inputs!$F$35)*Inputs!$F$37/1000</f>
-        <v>136.5</v>
+        <v>89.355</v>
       </c>
       <c r="F24" s="6" t="n">
         <f aca="false">Inputs!$G$34*(1-Inputs!$G$35)*Inputs!$G$37/1000</f>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="C25" s="6" t="n">
         <f aca="false">Inputs!$D$38*Inputs!$D$39</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" s="6" t="n">
         <f aca="false">Inputs!$E$38*Inputs!$E$39</f>
@@ -6478,7 +6478,7 @@
       </c>
       <c r="E25" s="6" t="n">
         <f aca="false">Inputs!$F$38*Inputs!$F$39</f>
-        <v>30</v>
+        <v>18.9</v>
       </c>
       <c r="F25" s="6" t="n">
         <f aca="false">Inputs!$G$38*Inputs!$G$39</f>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">Inputs!$D$45</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D26" s="6" t="n">
         <f aca="false">Inputs!$E$45</f>
@@ -6505,7 +6505,7 @@
       </c>
       <c r="E26" s="6" t="n">
         <f aca="false">Inputs!$F$45</f>
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F26" s="6" t="n">
         <f aca="false">Inputs!$G$45</f>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C27" s="35" t="n">
         <f aca="false">SUM(C19:C26)</f>
-        <v>91.82922</v>
+        <v>149.953848</v>
       </c>
       <c r="D27" s="35" t="n">
         <f aca="false">SUM(D19:D26)</f>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="E27" s="35" t="n">
         <f aca="false">SUM(E19:E26)</f>
-        <v>765.0088</v>
+        <v>483.83538</v>
       </c>
       <c r="F27" s="35" t="n">
         <f aca="false">SUM(F19:F26)</f>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">SUM(C19:C22)</f>
-        <v>52.19172</v>
+        <v>91.609848</v>
       </c>
       <c r="D28" s="33" t="n">
         <f aca="false">SUM(D19:D22)</f>
@@ -6557,7 +6557,7 @@
       </c>
       <c r="E28" s="33" t="n">
         <f aca="false">SUM(E19:E22)</f>
-        <v>513.7088</v>
+        <v>318.04038</v>
       </c>
       <c r="F28" s="33" t="n">
         <f aca="false">SUM(F19:F22)</f>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="C29" s="33" t="n">
         <f aca="false">SUM(C23:C25)</f>
-        <v>35.6375</v>
+        <v>52.344</v>
       </c>
       <c r="D29" s="33" t="n">
         <f aca="false">SUM(D23:D25)</f>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E29" s="33" t="n">
         <f aca="false">SUM(E23:E25)</f>
-        <v>231.3</v>
+        <v>153.795</v>
       </c>
       <c r="F29" s="33" t="n">
         <f aca="false">SUM(F23:F25)</f>
@@ -6599,7 +6599,7 @@
       </c>
       <c r="C30" s="36" t="n">
         <f aca="false">IF(C27=0,0,C28/C27)</f>
-        <v>0.56835634670533</v>
+        <v>0.610920287954198</v>
       </c>
       <c r="D30" s="36" t="n">
         <f aca="false">IF(D27=0,0,D28/D27)</f>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="E30" s="36" t="n">
         <f aca="false">IF(E27=0,0,E28/E27)</f>
-        <v>0.671507046716325</v>
+        <v>0.657331797439038</v>
       </c>
       <c r="F30" s="36" t="n">
         <f aca="false">IF(F27=0,0,F28/F27)</f>
@@ -6635,7 +6635,7 @@
       </c>
       <c r="C33" s="13" t="n">
         <f aca="false">Inputs!$D$48</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D33" s="13" t="n">
         <f aca="false">Inputs!$E$48</f>
@@ -6660,7 +6660,7 @@
       </c>
       <c r="C34" s="14" t="n">
         <f aca="false">Inputs!$D$49</f>
-        <v>0.48</v>
+        <v>0.5</v>
       </c>
       <c r="D34" s="14" t="n">
         <f aca="false">Inputs!$E$49</f>
@@ -6668,7 +6668,7 @@
       </c>
       <c r="E34" s="14" t="n">
         <f aca="false">Inputs!$F$49</f>
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="F34" s="14" t="n">
         <f aca="false">Inputs!$G$49</f>
@@ -6685,7 +6685,7 @@
       </c>
       <c r="C35" s="37" t="n">
         <f aca="false">C33*C34</f>
-        <v>6.72</v>
+        <v>7.5</v>
       </c>
       <c r="D35" s="37" t="n">
         <f aca="false">D33*D34</f>
@@ -6693,7 +6693,7 @@
       </c>
       <c r="E35" s="37" t="n">
         <f aca="false">E33*E34</f>
-        <v>16.5</v>
+        <v>15.95</v>
       </c>
       <c r="F35" s="37" t="n">
         <f aca="false">F33*F34</f>
@@ -6712,7 +6712,7 @@
       </c>
       <c r="C36" s="5" t="n">
         <f aca="false">Inputs!$D$50</f>
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D36" s="5" t="n">
         <f aca="false">Inputs!$E$50</f>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="E36" s="5" t="n">
         <f aca="false">Inputs!$F$50</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F36" s="5" t="n">
         <f aca="false">Inputs!$G$50</f>
@@ -6737,7 +6737,7 @@
       </c>
       <c r="C37" s="38" t="n">
         <f aca="false">C36*C34</f>
-        <v>10.56</v>
+        <v>10</v>
       </c>
       <c r="D37" s="38" t="n">
         <f aca="false">D36*D34</f>
@@ -6745,7 +6745,7 @@
       </c>
       <c r="E37" s="38" t="n">
         <f aca="false">E36*E34</f>
-        <v>24</v>
+        <v>17.4</v>
       </c>
       <c r="F37" s="38" t="n">
         <f aca="false">F36*F34</f>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="C38" s="35" t="n">
         <f aca="false">C35*C36</f>
-        <v>147.84</v>
+        <v>150</v>
       </c>
       <c r="D38" s="35" t="n">
         <f aca="false">D35*D36</f>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="E38" s="35" t="n">
         <f aca="false">E35*E36</f>
-        <v>660</v>
+        <v>478.5</v>
       </c>
       <c r="F38" s="35" t="n">
         <f aca="false">F35*F36</f>
@@ -6789,7 +6789,7 @@
       </c>
       <c r="C39" s="38" t="n">
         <f aca="false">C27</f>
-        <v>91.82922</v>
+        <v>149.953848</v>
       </c>
       <c r="D39" s="38" t="n">
         <f aca="false">D27</f>
@@ -6797,7 +6797,7 @@
       </c>
       <c r="E39" s="38" t="n">
         <f aca="false">E27</f>
-        <v>765.0088</v>
+        <v>483.83538</v>
       </c>
       <c r="F39" s="38" t="n">
         <f aca="false">F27</f>
@@ -6814,7 +6814,7 @@
       </c>
       <c r="C40" s="39" t="n">
         <f aca="false">IF(C38=0,0,C39/C38)</f>
-        <v>0.621139204545455</v>
+        <v>0.99969232</v>
       </c>
       <c r="D40" s="39" t="n">
         <f aca="false">IF(D38=0,0,D39/D38)</f>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="E40" s="39" t="n">
         <f aca="false">IF(E38=0,0,E39/E38)</f>
-        <v>1.15910424242424</v>
+        <v>1.01115021943574</v>
       </c>
       <c r="F40" s="39" t="n">
         <f aca="false">IF(F38=0,0,F39/F38)</f>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="C41" s="38" t="n">
         <f aca="false">IF(C35=0,0,C39/C35)</f>
-        <v>13.6650625</v>
+        <v>19.9938464</v>
       </c>
       <c r="D41" s="38" t="n">
         <f aca="false">IF(D35=0,0,D39/D35)</f>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="E41" s="38" t="n">
         <f aca="false">IF(E35=0,0,E39/E35)</f>
-        <v>46.3641696969697</v>
+        <v>30.3345065830721</v>
       </c>
       <c r="F41" s="38" t="n">
         <f aca="false">IF(F35=0,0,F39/F35)</f>
@@ -6866,7 +6866,7 @@
       </c>
       <c r="C42" s="5" t="n">
         <f aca="false">Inputs!$D$51</f>
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="D42" s="5" t="n">
         <f aca="false">Inputs!$E$51</f>
@@ -6874,7 +6874,7 @@
       </c>
       <c r="E42" s="5" t="n">
         <f aca="false">Inputs!$F$51</f>
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">Inputs!$G$51</f>
@@ -6891,7 +6891,7 @@
       </c>
       <c r="C43" s="5" t="n">
         <f aca="false">C35*C42+Inputs!$D$52*C38</f>
-        <v>95.2896</v>
+        <v>99.75</v>
       </c>
       <c r="D43" s="5" t="n">
         <f aca="false">D35*D42+Inputs!$E$52*D38</f>
@@ -6899,7 +6899,7 @@
       </c>
       <c r="E43" s="5" t="n">
         <f aca="false">E35*E42+Inputs!$F$52*E38</f>
-        <v>181.5</v>
+        <v>179.4375</v>
       </c>
       <c r="F43" s="5" t="n">
         <f aca="false">F35*F42+Inputs!$G$52*F38</f>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="C44" s="22" t="n">
         <f aca="false">IF(C38=0,0,1-C43/C38)</f>
-        <v>0.355454545454545</v>
+        <v>0.335</v>
       </c>
       <c r="D44" s="22" t="n">
         <f aca="false">IF(D38=0,0,1-D43/D38)</f>
@@ -6926,7 +6926,7 @@
       </c>
       <c r="E44" s="22" t="n">
         <f aca="false">IF(E38=0,0,1-E43/E38)</f>
-        <v>0.725</v>
+        <v>0.625</v>
       </c>
       <c r="F44" s="22" t="n">
         <f aca="false">IF(F38=0,0,1-F43/F38)</f>
@@ -6945,7 +6945,7 @@
       </c>
       <c r="C45" s="40" t="n">
         <f aca="false">IF(Inputs!$D$60*Inputs!$D$61=0,0,C36/(Inputs!$D$60*Inputs!$D$61))</f>
-        <v>2.29166666666667</v>
+        <v>2.08333333333333</v>
       </c>
       <c r="D45" s="40" t="n">
         <f aca="false">IF(Inputs!$E$60*Inputs!$E$61=0,0,D36/(Inputs!$E$60*Inputs!$E$61))</f>
@@ -6953,7 +6953,7 @@
       </c>
       <c r="E45" s="40" t="n">
         <f aca="false">IF(Inputs!$F$60*Inputs!$F$61=0,0,E36/(Inputs!$F$60*Inputs!$F$61))</f>
-        <v>1.6025641025641</v>
+        <v>1.20192307692308</v>
       </c>
       <c r="F45" s="40" t="n">
         <f aca="false">IF(Inputs!$G$60*Inputs!$G$61=0,0,F36/(Inputs!$G$60*Inputs!$G$61))</f>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C48" s="5" t="n">
         <f aca="false">Inputs!$D$67</f>
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D48" s="5" t="n">
         <f aca="false">Inputs!$E$67</f>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C49" s="5" t="n">
         <f aca="false">C48*(1+Inputs!$D$69)</f>
-        <v>72.5</v>
+        <v>92.8</v>
       </c>
       <c r="D49" s="5" t="n">
         <f aca="false">D48*(1+Inputs!$E$69)</f>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="E49" s="5" t="n">
         <f aca="false">E48*(1+Inputs!$F$69)</f>
-        <v>156</v>
+        <v>152.75</v>
       </c>
       <c r="F49" s="5" t="n">
         <f aca="false">F48*(1+Inputs!$G$69)</f>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="C50" s="38" t="n">
         <f aca="false">(C48+C49)/2</f>
-        <v>61.25</v>
+        <v>75.4</v>
       </c>
       <c r="D50" s="38" t="n">
         <f aca="false">(D48+D49)/2</f>
@@ -7043,7 +7043,7 @@
       </c>
       <c r="E50" s="38" t="n">
         <f aca="false">(E48+E49)/2</f>
-        <v>110.5</v>
+        <v>108.875</v>
       </c>
       <c r="F50" s="38" t="n">
         <f aca="false">(F48+F49)/2</f>
@@ -7062,7 +7062,7 @@
       </c>
       <c r="C51" s="5" t="n">
         <f aca="false">C49*(1+Inputs!$D$70)</f>
-        <v>94.25</v>
+        <v>122.496</v>
       </c>
       <c r="D51" s="5" t="n">
         <f aca="false">D49*(1+Inputs!$E$70)</f>
@@ -7070,7 +7070,7 @@
       </c>
       <c r="E51" s="5" t="n">
         <f aca="false">E49*(1+Inputs!$F$70)</f>
-        <v>273</v>
+        <v>274.95</v>
       </c>
       <c r="F51" s="5" t="n">
         <f aca="false">F49*(1+Inputs!$G$70)</f>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="C52" s="38" t="n">
         <f aca="false">(C49+C51)/2</f>
-        <v>83.375</v>
+        <v>107.648</v>
       </c>
       <c r="D52" s="38" t="n">
         <f aca="false">(D49+D51)/2</f>
@@ -7097,7 +7097,7 @@
       </c>
       <c r="E52" s="38" t="n">
         <f aca="false">(E49+E51)/2</f>
-        <v>214.5</v>
+        <v>213.85</v>
       </c>
       <c r="F52" s="38" t="n">
         <f aca="false">(F49+F51)/2</f>
@@ -7116,7 +7116,7 @@
       </c>
       <c r="C53" s="5" t="n">
         <f aca="false">C51*(1+Inputs!$D$71)</f>
-        <v>113.1</v>
+        <v>144.54528</v>
       </c>
       <c r="D53" s="5" t="n">
         <f aca="false">D51*(1+Inputs!$E$71)</f>
@@ -7124,7 +7124,7 @@
       </c>
       <c r="E53" s="5" t="n">
         <f aca="false">E51*(1+Inputs!$F$71)</f>
-        <v>395.85</v>
+        <v>406.926</v>
       </c>
       <c r="F53" s="5" t="n">
         <f aca="false">F51*(1+Inputs!$G$71)</f>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="C54" s="38" t="n">
         <f aca="false">(C51+C53)/2</f>
-        <v>103.675</v>
+        <v>133.52064</v>
       </c>
       <c r="D54" s="38" t="n">
         <f aca="false">(D51+D53)/2</f>
@@ -7151,7 +7151,7 @@
       </c>
       <c r="E54" s="38" t="n">
         <f aca="false">(E51+E53)/2</f>
-        <v>334.425</v>
+        <v>340.938</v>
       </c>
       <c r="F54" s="38" t="n">
         <f aca="false">(F51+F53)/2</f>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="C55" s="5" t="n">
         <f aca="false">C53*(1+Inputs!$D$72)</f>
-        <v>126.672</v>
+        <v>158.999808</v>
       </c>
       <c r="D55" s="5" t="n">
         <f aca="false">D53*(1+Inputs!$E$72)</f>
@@ -7178,7 +7178,7 @@
       </c>
       <c r="E55" s="5" t="n">
         <f aca="false">E53*(1+Inputs!$F$72)</f>
-        <v>514.605</v>
+        <v>537.14232</v>
       </c>
       <c r="F55" s="5" t="n">
         <f aca="false">F53*(1+Inputs!$G$72)</f>
@@ -7197,7 +7197,7 @@
       </c>
       <c r="C56" s="38" t="n">
         <f aca="false">(C53+C55)/2</f>
-        <v>119.886</v>
+        <v>151.772544</v>
       </c>
       <c r="D56" s="38" t="n">
         <f aca="false">(D53+D55)/2</f>
@@ -7205,7 +7205,7 @@
       </c>
       <c r="E56" s="38" t="n">
         <f aca="false">(E53+E55)/2</f>
-        <v>455.2275</v>
+        <v>472.03416</v>
       </c>
       <c r="F56" s="38" t="n">
         <f aca="false">(F53+F55)/2</f>
@@ -7224,7 +7224,7 @@
       </c>
       <c r="C57" s="39" t="n">
         <f aca="false">IF(C56=0,0,C27/C56)</f>
-        <v>0.765971172613983</v>
+        <v>0.988016963068103</v>
       </c>
       <c r="D57" s="39" t="n">
         <f aca="false">IF(D56=0,0,D27/D56)</f>
@@ -7232,7 +7232,7 @@
       </c>
       <c r="E57" s="39" t="n">
         <f aca="false">IF(E56=0,0,E27/E56)</f>
-        <v>1.68049777309148</v>
+        <v>1.02500077536761</v>
       </c>
       <c r="F57" s="39" t="n">
         <f aca="false">IF(F56=0,0,F27/F56)</f>
@@ -7285,7 +7285,7 @@
       </c>
       <c r="C61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",C19/$B61)</f>
-        <v>5.80608</v>
+        <v>10.0606628571429</v>
       </c>
       <c r="D61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",D19/$B61)</f>
@@ -7293,7 +7293,7 @@
       </c>
       <c r="E61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",E19/$B61)</f>
-        <v>46.4310857142857</v>
+        <v>31.8587657142857</v>
       </c>
       <c r="F61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",F19/$B61)</f>
@@ -7313,7 +7313,7 @@
       </c>
       <c r="C62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",C20/$B62)</f>
-        <v>2.1812</v>
+        <v>3.8342304</v>
       </c>
       <c r="D62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",D20/$B62)</f>
@@ -7321,7 +7321,7 @@
       </c>
       <c r="E62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",E20/$B62)</f>
-        <v>22.464</v>
+        <v>13.8138</v>
       </c>
       <c r="F62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",F20/$B62)</f>
@@ -7341,7 +7341,7 @@
       </c>
       <c r="C63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",C21/$B63)</f>
-        <v>2.08413333333333</v>
+        <v>3.596</v>
       </c>
       <c r="D63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",D21/$B63)</f>
@@ -7349,7 +7349,7 @@
       </c>
       <c r="E63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",E21/$B63)</f>
-        <v>28.9777777777778</v>
+        <v>16.864</v>
       </c>
       <c r="F63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",F21/$B63)</f>
@@ -7369,7 +7369,7 @@
       </c>
       <c r="C64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",C22/$B64)</f>
-        <v>2.13818181818182</v>
+        <v>3.84872727272727</v>
       </c>
       <c r="D64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",D22/$B64)</f>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="E64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",E22/$B64)</f>
-        <v>23.7381818181818</v>
+        <v>13.1956363636364</v>
       </c>
       <c r="F64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",F22/$B64)</f>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="C65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",C23/$B65)</f>
-        <v>0.783870967741936</v>
+        <v>1.0306064516129</v>
       </c>
       <c r="D65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",D23/$B65)</f>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",E23/$B65)</f>
-        <v>4.18064516129032</v>
+        <v>2.93806451612903</v>
       </c>
       <c r="F65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",F23/$B65)</f>
@@ -7425,7 +7425,7 @@
       </c>
       <c r="C66" s="42" t="n">
         <f aca="false">IF($B66=0,"n/a",C24/$B66)</f>
-        <v>21.4875</v>
+        <v>33.3696</v>
       </c>
       <c r="D66" s="42" t="n">
         <f aca="false">IF($B66=0,"n/a",D24/$B66)</f>
@@ -7433,7 +7433,7 @@
       </c>
       <c r="E66" s="42" t="n">
         <f aca="false">IF($B66=0,"n/a",E24/$B66)</f>
-        <v>136.5</v>
+        <v>89.355</v>
       </c>
       <c r="F66" s="42" t="n">
         <f aca="false">IF($B66=0,"n/a",F24/$B66)</f>
@@ -7453,7 +7453,7 @@
       </c>
       <c r="C67" s="42" t="n">
         <f aca="false">IF($B67=0,"n/a",C25/$B67)</f>
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="D67" s="42" t="n">
         <f aca="false">IF($B67=0,"n/a",D25/$B67)</f>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="E67" s="42" t="n">
         <f aca="false">IF($B67=0,"n/a",E25/$B67)</f>
-        <v>75</v>
+        <v>47.25</v>
       </c>
       <c r="F67" s="42" t="n">
         <f aca="false">IF($B67=0,"n/a",F25/$B67)</f>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="C68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",C26/$B68)</f>
-        <v>3.07692307692308</v>
+        <v>4.61538461538462</v>
       </c>
       <c r="D68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",D26/$B68)</f>
@@ -7489,7 +7489,7 @@
       </c>
       <c r="E68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",E26/$B68)</f>
-        <v>15.3846153846154</v>
+        <v>9.23076923076923</v>
       </c>
       <c r="F68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",F26/$B68)</f>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="C69" s="42" t="n">
         <f aca="false">C27/$B69</f>
-        <v>2.51586904109589</v>
+        <v>4.10832460273973</v>
       </c>
       <c r="D69" s="42" t="n">
         <f aca="false">D27/$B69</f>
@@ -7518,7 +7518,7 @@
       </c>
       <c r="E69" s="42" t="n">
         <f aca="false">E27/$B69</f>
-        <v>20.9591452054795</v>
+        <v>13.2557638356164</v>
       </c>
       <c r="F69" s="42" t="n">
         <f aca="false">F27/$B69</f>
@@ -7797,7 +7797,7 @@
       </c>
       <c r="C6" s="31" t="n">
         <f aca="false">Inputs!$D$9*Inputs!$D$17*1000</f>
-        <v>5760</v>
+        <v>7920</v>
       </c>
       <c r="D6" s="31" t="n">
         <f aca="false">Inputs!$E$9*Inputs!$E$17*1000</f>
@@ -7805,7 +7805,7 @@
       </c>
       <c r="E6" s="31" t="n">
         <f aca="false">Inputs!$F$9*Inputs!$F$17*1000</f>
-        <v>16000</v>
+        <v>14820</v>
       </c>
       <c r="F6" s="31" t="n">
         <f aca="false">Inputs!$G$9*Inputs!$G$17*1000</f>
@@ -7824,7 +7824,7 @@
       </c>
       <c r="C7" s="31" t="n">
         <f aca="false">Inputs!$D$10*Inputs!$D$18*1000</f>
-        <v>1140</v>
+        <v>1482</v>
       </c>
       <c r="D7" s="31" t="n">
         <f aca="false">Inputs!$E$10*Inputs!$E$18*1000</f>
@@ -7832,7 +7832,7 @@
       </c>
       <c r="E7" s="31" t="n">
         <f aca="false">Inputs!$F$10*Inputs!$F$18*1000</f>
-        <v>3900</v>
+        <v>3276</v>
       </c>
       <c r="F7" s="31" t="n">
         <f aca="false">Inputs!$G$10*Inputs!$G$18*1000</f>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="C8" s="31" t="n">
         <f aca="false">Inputs!$D$11*Inputs!$D$19*1000</f>
-        <v>232</v>
+        <v>261</v>
       </c>
       <c r="D8" s="31" t="n">
         <f aca="false">Inputs!$E$11*Inputs!$E$19*1000</f>
@@ -7857,7 +7857,7 @@
       </c>
       <c r="E8" s="31" t="n">
         <f aca="false">Inputs!$F$11*Inputs!$F$19*1000</f>
-        <v>640</v>
+        <v>527</v>
       </c>
       <c r="F8" s="31" t="n">
         <f aca="false">Inputs!$G$11*Inputs!$G$19*1000</f>
@@ -7874,7 +7874,7 @@
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">Inputs!$D$6*Inputs!$D$13</f>
-        <v>25.2</v>
+        <v>29.64</v>
       </c>
       <c r="D9" s="32" t="n">
         <f aca="false">Inputs!$E$6*Inputs!$E$13</f>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="E9" s="32" t="n">
         <f aca="false">Inputs!$F$6*Inputs!$F$13</f>
-        <v>42.32</v>
+        <v>39.6</v>
       </c>
       <c r="F9" s="32" t="n">
         <f aca="false">Inputs!$G$6*Inputs!$G$13</f>
@@ -7901,7 +7901,7 @@
       </c>
       <c r="C10" s="32" t="n">
         <f aca="false">Inputs!$D$7*Inputs!$D$14</f>
-        <v>71.75</v>
+        <v>88.2</v>
       </c>
       <c r="D10" s="32" t="n">
         <f aca="false">Inputs!$E$7*Inputs!$E$14</f>
@@ -7909,7 +7909,7 @@
       </c>
       <c r="E10" s="32" t="n">
         <f aca="false">Inputs!$F$7*Inputs!$F$14</f>
-        <v>144</v>
+        <v>126.5</v>
       </c>
       <c r="F10" s="32" t="n">
         <f aca="false">Inputs!$G$7*Inputs!$G$14</f>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="C11" s="32" t="n">
         <f aca="false">Inputs!$D$8*Inputs!$D$15</f>
-        <v>115.5</v>
+        <v>155</v>
       </c>
       <c r="D11" s="32" t="n">
         <f aca="false">Inputs!$E$8*Inputs!$E$15</f>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="E11" s="32" t="n">
         <f aca="false">Inputs!$F$8*Inputs!$F$15</f>
-        <v>326</v>
+        <v>288</v>
       </c>
       <c r="F11" s="32" t="n">
         <f aca="false">Inputs!$G$8*Inputs!$G$15</f>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="C12" s="33" t="n">
         <f aca="false">C9*C6/1000</f>
-        <v>145.152</v>
+        <v>234.7488</v>
       </c>
       <c r="D12" s="33" t="n">
         <f aca="false">D9*D6/1000</f>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="E12" s="33" t="n">
         <f aca="false">E9*E6/1000</f>
-        <v>677.12</v>
+        <v>586.872</v>
       </c>
       <c r="F12" s="33" t="n">
         <f aca="false">F9*F6/1000</f>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="C13" s="33" t="n">
         <f aca="false">C10*C7/1000</f>
-        <v>81.795</v>
+        <v>130.7124</v>
       </c>
       <c r="D13" s="33" t="n">
         <f aca="false">D10*D7/1000</f>
@@ -7986,7 +7986,7 @@
       </c>
       <c r="E13" s="33" t="n">
         <f aca="false">E10*E7/1000</f>
-        <v>561.6</v>
+        <v>414.414</v>
       </c>
       <c r="F13" s="33" t="n">
         <f aca="false">F10*F7/1000</f>
@@ -8003,7 +8003,7 @@
       </c>
       <c r="C14" s="33" t="n">
         <f aca="false">C11*C8/1000</f>
-        <v>26.796</v>
+        <v>40.455</v>
       </c>
       <c r="D14" s="33" t="n">
         <f aca="false">D11*D8/1000</f>
@@ -8011,7 +8011,7 @@
       </c>
       <c r="E14" s="33" t="n">
         <f aca="false">E11*E8/1000</f>
-        <v>208.64</v>
+        <v>151.776</v>
       </c>
       <c r="F14" s="33" t="n">
         <f aca="false">F11*F8/1000</f>
@@ -8028,7 +8028,7 @@
       </c>
       <c r="C15" s="6" t="n">
         <f aca="false">Inputs!$D$28*Inputs!$D$29*Inputs!$D$30*1000</f>
-        <v>98</v>
+        <v>151.2</v>
       </c>
       <c r="D15" s="6" t="n">
         <f aca="false">Inputs!$E$28*Inputs!$E$29*Inputs!$E$30*1000</f>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="E15" s="6" t="n">
         <f aca="false">Inputs!$F$28*Inputs!$F$29*Inputs!$F$30*1000</f>
-        <v>544</v>
+        <v>403.2</v>
       </c>
       <c r="F15" s="6" t="n">
         <f aca="false">Inputs!$G$28*Inputs!$G$29*Inputs!$G$30*1000</f>
@@ -8055,7 +8055,7 @@
       </c>
       <c r="C16" s="34" t="n">
         <f aca="false">SUM(C12:C15)</f>
-        <v>351.743</v>
+        <v>557.1162</v>
       </c>
       <c r="D16" s="34" t="n">
         <f aca="false">SUM(D12:D15)</f>
@@ -8063,7 +8063,7 @@
       </c>
       <c r="E16" s="34" t="n">
         <f aca="false">SUM(E12:E15)</f>
-        <v>1991.36</v>
+        <v>1556.262</v>
       </c>
       <c r="F16" s="34" t="n">
         <f aca="false">SUM(F12:F15)</f>
@@ -8091,7 +8091,7 @@
       </c>
       <c r="C19" s="6" t="n">
         <f aca="false">C12*Inputs!$D$21</f>
-        <v>52.25472</v>
+        <v>98.594496</v>
       </c>
       <c r="D19" s="6" t="n">
         <f aca="false">D12*Inputs!$E$21</f>
@@ -8099,7 +8099,7 @@
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">E12*Inputs!$F$21</f>
-        <v>325.0176</v>
+        <v>269.96112</v>
       </c>
       <c r="F19" s="6" t="n">
         <f aca="false">F12*Inputs!$G$21</f>
@@ -8118,7 +8118,7 @@
       </c>
       <c r="C20" s="6" t="n">
         <f aca="false">C13*Inputs!$D$23</f>
-        <v>10.63335</v>
+        <v>20.913984</v>
       </c>
       <c r="D20" s="6" t="n">
         <f aca="false">D13*Inputs!$E$23</f>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="E20" s="6" t="n">
         <f aca="false">E13*Inputs!$F$23</f>
-        <v>134.784</v>
+        <v>87.02694</v>
       </c>
       <c r="F20" s="6" t="n">
         <f aca="false">F13*Inputs!$G$23</f>
@@ -8143,7 +8143,7 @@
       </c>
       <c r="C21" s="6" t="n">
         <f aca="false">C14*Inputs!$D$25</f>
-        <v>1.3398</v>
+        <v>2.4273</v>
       </c>
       <c r="D21" s="6" t="n">
         <f aca="false">D14*Inputs!$E$25</f>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">E14*Inputs!$F$25</f>
-        <v>25.0368</v>
+        <v>15.1776</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">F14*Inputs!$G$25</f>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="C22" s="6" t="n">
         <f aca="false">C15*Inputs!$D$31</f>
-        <v>29.4</v>
+        <v>60.48</v>
       </c>
       <c r="D22" s="6" t="n">
         <f aca="false">D15*Inputs!$E$31</f>
@@ -8176,7 +8176,7 @@
       </c>
       <c r="E22" s="6" t="n">
         <f aca="false">E15*Inputs!$F$31</f>
-        <v>244.8</v>
+        <v>173.376</v>
       </c>
       <c r="F22" s="6" t="n">
         <f aca="false">F15*Inputs!$G$31</f>
@@ -8195,7 +8195,7 @@
       </c>
       <c r="C23" s="6" t="n">
         <f aca="false">Inputs!$D$41*Inputs!$D$42*Inputs!$D$43*12/1000</f>
-        <v>3.744</v>
+        <v>7.2</v>
       </c>
       <c r="D23" s="6" t="n">
         <f aca="false">Inputs!$E$41*Inputs!$E$42*Inputs!$E$43*12/1000</f>
@@ -8203,7 +8203,7 @@
       </c>
       <c r="E23" s="6" t="n">
         <f aca="false">Inputs!$F$41*Inputs!$F$42*Inputs!$F$43*12/1000</f>
-        <v>30.24</v>
+        <v>22.932</v>
       </c>
       <c r="F23" s="6" t="n">
         <f aca="false">Inputs!$G$41*Inputs!$G$42*Inputs!$G$43*12/1000</f>
@@ -8276,7 +8276,7 @@
       </c>
       <c r="C26" s="6" t="n">
         <f aca="false">Inputs!$D$46</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D26" s="6" t="n">
         <f aca="false">Inputs!$E$46</f>
@@ -8284,7 +8284,7 @@
       </c>
       <c r="E26" s="6" t="n">
         <f aca="false">Inputs!$F$46</f>
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F26" s="6" t="n">
         <f aca="false">Inputs!$G$46</f>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="C27" s="35" t="n">
         <f aca="false">SUM(C19:C26)</f>
-        <v>101.37187</v>
+        <v>199.61578</v>
       </c>
       <c r="D27" s="35" t="n">
         <f aca="false">SUM(D19:D26)</f>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="E27" s="35" t="n">
         <f aca="false">SUM(E19:E26)</f>
-        <v>779.8784</v>
+        <v>584.47366</v>
       </c>
       <c r="F27" s="35" t="n">
         <f aca="false">SUM(F19:F26)</f>
@@ -8328,7 +8328,7 @@
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">SUM(C19:C22)</f>
-        <v>93.62787</v>
+        <v>182.41578</v>
       </c>
       <c r="D28" s="33" t="n">
         <f aca="false">SUM(D19:D22)</f>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="E28" s="33" t="n">
         <f aca="false">SUM(E19:E22)</f>
-        <v>729.6384</v>
+        <v>545.54166</v>
       </c>
       <c r="F28" s="33" t="n">
         <f aca="false">SUM(F19:F22)</f>
@@ -8353,7 +8353,7 @@
       </c>
       <c r="C29" s="33" t="n">
         <f aca="false">SUM(C23:C25)</f>
-        <v>3.744</v>
+        <v>7.2</v>
       </c>
       <c r="D29" s="33" t="n">
         <f aca="false">SUM(D23:D25)</f>
@@ -8361,7 +8361,7 @@
       </c>
       <c r="E29" s="33" t="n">
         <f aca="false">SUM(E23:E25)</f>
-        <v>30.24</v>
+        <v>22.932</v>
       </c>
       <c r="F29" s="33" t="n">
         <f aca="false">SUM(F23:F25)</f>
@@ -8378,7 +8378,7 @@
       </c>
       <c r="C30" s="36" t="n">
         <f aca="false">IF(C27=0,0,C28/C27)</f>
-        <v>0.923607998944875</v>
+        <v>0.913834467395313</v>
       </c>
       <c r="D30" s="36" t="n">
         <f aca="false">IF(D27=0,0,D28/D27)</f>
@@ -8386,7 +8386,7 @@
       </c>
       <c r="E30" s="36" t="n">
         <f aca="false">IF(E27=0,0,E28/E27)</f>
-        <v>0.935579700630252</v>
+        <v>0.933389641545181</v>
       </c>
       <c r="F30" s="36" t="n">
         <f aca="false">IF(F27=0,0,F28/F27)</f>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="C33" s="13" t="n">
         <f aca="false">Inputs!$D$54</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D33" s="13" t="n">
         <f aca="false">Inputs!$E$54</f>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="C34" s="14" t="n">
         <f aca="false">Inputs!$D$55</f>
-        <v>0.48</v>
+        <v>0.52</v>
       </c>
       <c r="D34" s="14" t="n">
         <f aca="false">Inputs!$E$55</f>
@@ -8447,7 +8447,7 @@
       </c>
       <c r="E34" s="14" t="n">
         <f aca="false">Inputs!$F$55</f>
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="F34" s="14" t="n">
         <f aca="false">Inputs!$G$55</f>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="C35" s="37" t="n">
         <f aca="false">C33*C34</f>
-        <v>7.2</v>
+        <v>8.32</v>
       </c>
       <c r="D35" s="37" t="n">
         <f aca="false">D33*D34</f>
@@ -8472,7 +8472,7 @@
       </c>
       <c r="E35" s="37" t="n">
         <f aca="false">E33*E34</f>
-        <v>15</v>
+        <v>14.5</v>
       </c>
       <c r="F35" s="37" t="n">
         <f aca="false">F33*F34</f>
@@ -8491,7 +8491,7 @@
       </c>
       <c r="C36" s="5" t="n">
         <f aca="false">Inputs!$D$56</f>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D36" s="5" t="n">
         <f aca="false">Inputs!$E$56</f>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="E36" s="5" t="n">
         <f aca="false">Inputs!$F$56</f>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F36" s="5" t="n">
         <f aca="false">Inputs!$G$56</f>
@@ -8516,7 +8516,7 @@
       </c>
       <c r="C37" s="38" t="n">
         <f aca="false">C36*C34</f>
-        <v>12</v>
+        <v>12.48</v>
       </c>
       <c r="D37" s="38" t="n">
         <f aca="false">D36*D34</f>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="E37" s="38" t="n">
         <f aca="false">E36*E34</f>
-        <v>27</v>
+        <v>23.2</v>
       </c>
       <c r="F37" s="38" t="n">
         <f aca="false">F36*F34</f>
@@ -8543,7 +8543,7 @@
       </c>
       <c r="C38" s="35" t="n">
         <f aca="false">C35*C36</f>
-        <v>180</v>
+        <v>199.68</v>
       </c>
       <c r="D38" s="35" t="n">
         <f aca="false">D35*D36</f>
@@ -8551,7 +8551,7 @@
       </c>
       <c r="E38" s="35" t="n">
         <f aca="false">E35*E36</f>
-        <v>675</v>
+        <v>580</v>
       </c>
       <c r="F38" s="35" t="n">
         <f aca="false">F35*F36</f>
@@ -8568,7 +8568,7 @@
       </c>
       <c r="C39" s="38" t="n">
         <f aca="false">C27</f>
-        <v>101.37187</v>
+        <v>199.61578</v>
       </c>
       <c r="D39" s="38" t="n">
         <f aca="false">D27</f>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="E39" s="38" t="n">
         <f aca="false">E27</f>
-        <v>779.8784</v>
+        <v>584.47366</v>
       </c>
       <c r="F39" s="38" t="n">
         <f aca="false">F27</f>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="C40" s="39" t="n">
         <f aca="false">IF(C38=0,0,C39/C38)</f>
-        <v>0.563177055555556</v>
+        <v>0.999678385416667</v>
       </c>
       <c r="D40" s="39" t="n">
         <f aca="false">IF(D38=0,0,D39/D38)</f>
@@ -8601,7 +8601,7 @@
       </c>
       <c r="E40" s="39" t="n">
         <f aca="false">IF(E38=0,0,E39/E38)</f>
-        <v>1.15537540740741</v>
+        <v>1.00771320689655</v>
       </c>
       <c r="F40" s="39" t="n">
         <f aca="false">IF(F38=0,0,F39/F38)</f>
@@ -8620,7 +8620,7 @@
       </c>
       <c r="C41" s="38" t="n">
         <f aca="false">IF(C35=0,0,C39/C35)</f>
-        <v>14.0794263888889</v>
+        <v>23.99228125</v>
       </c>
       <c r="D41" s="38" t="n">
         <f aca="false">IF(D35=0,0,D39/D35)</f>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="E41" s="38" t="n">
         <f aca="false">IF(E35=0,0,E39/E35)</f>
-        <v>51.9918933333333</v>
+        <v>40.3085282758621</v>
       </c>
       <c r="F41" s="38" t="n">
         <f aca="false">IF(F35=0,0,F39/F35)</f>
@@ -8645,7 +8645,7 @@
       </c>
       <c r="C42" s="5" t="n">
         <f aca="false">Inputs!$D$57</f>
-        <v>13.3</v>
+        <v>12.5</v>
       </c>
       <c r="D42" s="5" t="n">
         <f aca="false">Inputs!$E$57</f>
@@ -8653,7 +8653,7 @@
       </c>
       <c r="E42" s="5" t="n">
         <f aca="false">Inputs!$F$57</f>
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">Inputs!$G$57</f>
@@ -8670,7 +8670,7 @@
       </c>
       <c r="C43" s="5" t="n">
         <f aca="false">C35*C42+Inputs!$D$58*C38</f>
-        <v>102.96</v>
+        <v>111.9872</v>
       </c>
       <c r="D43" s="5" t="n">
         <f aca="false">D35*D42+Inputs!$E$58*D38</f>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="E43" s="5" t="n">
         <f aca="false">E35*E42+Inputs!$F$58*E38</f>
-        <v>166.875</v>
+        <v>166.75</v>
       </c>
       <c r="F43" s="5" t="n">
         <f aca="false">F35*F42+Inputs!$G$58*F38</f>
@@ -8697,7 +8697,7 @@
       </c>
       <c r="C44" s="22" t="n">
         <f aca="false">IF(C38=0,0,1-C43/C38)</f>
-        <v>0.428</v>
+        <v>0.439166666666667</v>
       </c>
       <c r="D44" s="22" t="n">
         <f aca="false">IF(D38=0,0,1-D43/D38)</f>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="E44" s="22" t="n">
         <f aca="false">IF(E38=0,0,1-E43/E38)</f>
-        <v>0.752777777777778</v>
+        <v>0.7125</v>
       </c>
       <c r="F44" s="22" t="n">
         <f aca="false">IF(F38=0,0,1-F43/F38)</f>
@@ -8724,7 +8724,7 @@
       </c>
       <c r="C45" s="40" t="n">
         <f aca="false">IF(Inputs!$D$60*Inputs!$D$61=0,0,C36/(Inputs!$D$60*Inputs!$D$61))</f>
-        <v>2.60416666666667</v>
+        <v>2.5</v>
       </c>
       <c r="D45" s="40" t="n">
         <f aca="false">IF(Inputs!$E$60*Inputs!$E$61=0,0,D36/(Inputs!$E$60*Inputs!$E$61))</f>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="E45" s="40" t="n">
         <f aca="false">IF(Inputs!$F$60*Inputs!$F$61=0,0,E36/(Inputs!$F$60*Inputs!$F$61))</f>
-        <v>1.80288461538462</v>
+        <v>1.6025641025641</v>
       </c>
       <c r="F45" s="40" t="n">
         <f aca="false">IF(Inputs!$G$60*Inputs!$G$61=0,0,F36/(Inputs!$G$60*Inputs!$G$61))</f>
@@ -8762,7 +8762,7 @@
       </c>
       <c r="C48" s="5" t="n">
         <f aca="false">Inputs!$D$68</f>
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="D48" s="5" t="n">
         <f aca="false">Inputs!$E$68</f>
@@ -8787,7 +8787,7 @@
       </c>
       <c r="C49" s="5" t="n">
         <f aca="false">C48*(1+Inputs!$D$73)</f>
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="D49" s="5" t="n">
         <f aca="false">D48*(1+Inputs!$E$73)</f>
@@ -8795,7 +8795,7 @@
       </c>
       <c r="E49" s="5" t="n">
         <f aca="false">E48*(1+Inputs!$F$73)</f>
-        <v>231</v>
+        <v>225.5</v>
       </c>
       <c r="F49" s="5" t="n">
         <f aca="false">F48*(1+Inputs!$G$73)</f>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="C50" s="38" t="n">
         <f aca="false">(C48+C49)/2</f>
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="D50" s="38" t="n">
         <f aca="false">(D48+D49)/2</f>
@@ -8822,7 +8822,7 @@
       </c>
       <c r="E50" s="38" t="n">
         <f aca="false">(E48+E49)/2</f>
-        <v>170.5</v>
+        <v>167.75</v>
       </c>
       <c r="F50" s="38" t="n">
         <f aca="false">(F48+F49)/2</f>
@@ -8841,7 +8841,7 @@
       </c>
       <c r="C51" s="5" t="n">
         <f aca="false">C49*(1+Inputs!$D$74)</f>
-        <v>145.18</v>
+        <v>171.12</v>
       </c>
       <c r="D51" s="5" t="n">
         <f aca="false">D49*(1+Inputs!$E$74)</f>
@@ -8849,7 +8849,7 @@
       </c>
       <c r="E51" s="5" t="n">
         <f aca="false">E49*(1+Inputs!$F$74)</f>
-        <v>369.6</v>
+        <v>360.8</v>
       </c>
       <c r="F51" s="5" t="n">
         <f aca="false">F49*(1+Inputs!$G$74)</f>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="C52" s="38" t="n">
         <f aca="false">(C49+C51)/2</f>
-        <v>132.09</v>
+        <v>154.56</v>
       </c>
       <c r="D52" s="38" t="n">
         <f aca="false">(D49+D51)/2</f>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="E52" s="38" t="n">
         <f aca="false">(E49+E51)/2</f>
-        <v>300.3</v>
+        <v>293.15</v>
       </c>
       <c r="F52" s="38" t="n">
         <f aca="false">(F49+F51)/2</f>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="C53" s="5" t="n">
         <f aca="false">C51*(1+Inputs!$D$75)</f>
-        <v>162.6016</v>
+        <v>195.0768</v>
       </c>
       <c r="D53" s="5" t="n">
         <f aca="false">D51*(1+Inputs!$E$75)</f>
@@ -8903,7 +8903,7 @@
       </c>
       <c r="E53" s="5" t="n">
         <f aca="false">E51*(1+Inputs!$F$75)</f>
-        <v>498.96</v>
+        <v>497.904</v>
       </c>
       <c r="F53" s="5" t="n">
         <f aca="false">F51*(1+Inputs!$G$75)</f>
@@ -8922,7 +8922,7 @@
       </c>
       <c r="C54" s="38" t="n">
         <f aca="false">(C51+C53)/2</f>
-        <v>153.8908</v>
+        <v>183.0984</v>
       </c>
       <c r="D54" s="38" t="n">
         <f aca="false">(D51+D53)/2</f>
@@ -8930,7 +8930,7 @@
       </c>
       <c r="E54" s="38" t="n">
         <f aca="false">(E51+E53)/2</f>
-        <v>434.28</v>
+        <v>429.352</v>
       </c>
       <c r="F54" s="38" t="n">
         <f aca="false">(F51+F53)/2</f>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="C55" s="5" t="n">
         <f aca="false">C53*(1+Inputs!$D$76)</f>
-        <v>172.357696</v>
+        <v>210.682944</v>
       </c>
       <c r="D55" s="5" t="n">
         <f aca="false">D53*(1+Inputs!$E$76)</f>
@@ -8957,7 +8957,7 @@
       </c>
       <c r="E55" s="5" t="n">
         <f aca="false">E53*(1+Inputs!$F$76)</f>
-        <v>638.6688</v>
+        <v>637.31712</v>
       </c>
       <c r="F55" s="5" t="n">
         <f aca="false">F53*(1+Inputs!$G$76)</f>
@@ -8976,7 +8976,7 @@
       </c>
       <c r="C56" s="38" t="n">
         <f aca="false">(C53+C55)/2</f>
-        <v>167.479648</v>
+        <v>202.879872</v>
       </c>
       <c r="D56" s="38" t="n">
         <f aca="false">(D53+D55)/2</f>
@@ -8984,7 +8984,7 @@
       </c>
       <c r="E56" s="38" t="n">
         <f aca="false">(E53+E55)/2</f>
-        <v>568.8144</v>
+        <v>567.61056</v>
       </c>
       <c r="F56" s="38" t="n">
         <f aca="false">(F53+F55)/2</f>
@@ -9003,7 +9003,7 @@
       </c>
       <c r="C57" s="39" t="n">
         <f aca="false">IF(C56=0,0,C27/C56)</f>
-        <v>0.605278738106734</v>
+        <v>0.983911208303601</v>
       </c>
       <c r="D57" s="39" t="n">
         <f aca="false">IF(D56=0,0,D27/D56)</f>
@@ -9011,7 +9011,7 @@
       </c>
       <c r="E57" s="39" t="n">
         <f aca="false">IF(E56=0,0,E27/E56)</f>
-        <v>1.37105952310631</v>
+        <v>1.02970892578179</v>
       </c>
       <c r="F57" s="39" t="n">
         <f aca="false">IF(F56=0,0,F27/F56)</f>
@@ -9064,7 +9064,7 @@
       </c>
       <c r="C61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",C19/$B61)</f>
-        <v>2.37521454545455</v>
+        <v>4.481568</v>
       </c>
       <c r="D61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",D19/$B61)</f>
@@ -9072,7 +9072,7 @@
       </c>
       <c r="E61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",E19/$B61)</f>
-        <v>14.7735272727273</v>
+        <v>12.27096</v>
       </c>
       <c r="F61" s="42" t="n">
         <f aca="false">IF($B61=0,"n/a",F19/$B61)</f>
@@ -9092,7 +9092,7 @@
       </c>
       <c r="C62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",C20/$B62)</f>
-        <v>1.25098235294118</v>
+        <v>2.46046870588235</v>
       </c>
       <c r="D62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",D20/$B62)</f>
@@ -9100,7 +9100,7 @@
       </c>
       <c r="E62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",E20/$B62)</f>
-        <v>15.8569411764706</v>
+        <v>10.2384635294118</v>
       </c>
       <c r="F62" s="42" t="n">
         <f aca="false">IF($B62=0,"n/a",F20/$B62)</f>
@@ -9120,7 +9120,7 @@
       </c>
       <c r="C63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",C21/$B63)</f>
-        <v>1.67475</v>
+        <v>3.034125</v>
       </c>
       <c r="D63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",D21/$B63)</f>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="E63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",E21/$B63)</f>
-        <v>31.296</v>
+        <v>18.972</v>
       </c>
       <c r="F63" s="42" t="n">
         <f aca="false">IF($B63=0,"n/a",F21/$B63)</f>
@@ -9148,7 +9148,7 @@
       </c>
       <c r="C64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",C22/$B64)</f>
-        <v>1.68</v>
+        <v>3.456</v>
       </c>
       <c r="D64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",D22/$B64)</f>
@@ -9156,7 +9156,7 @@
       </c>
       <c r="E64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",E22/$B64)</f>
-        <v>13.9885714285714</v>
+        <v>9.9072</v>
       </c>
       <c r="F64" s="42" t="n">
         <f aca="false">IF($B64=0,"n/a",F22/$B64)</f>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="C65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",C23/$B65)</f>
-        <v>0.680727272727273</v>
+        <v>1.30909090909091</v>
       </c>
       <c r="D65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",D23/$B65)</f>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="E65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",E23/$B65)</f>
-        <v>5.49818181818182</v>
+        <v>4.16945454545455</v>
       </c>
       <c r="F65" s="42" t="n">
         <f aca="false">IF($B65=0,"n/a",F23/$B65)</f>
@@ -9260,7 +9260,7 @@
       </c>
       <c r="C68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",C26/$B68)</f>
-        <v>1.48148148148148</v>
+        <v>3.7037037037037</v>
       </c>
       <c r="D68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",D26/$B68)</f>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="E68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",E26/$B68)</f>
-        <v>7.40740740740741</v>
+        <v>5.92592592592593</v>
       </c>
       <c r="F68" s="42" t="n">
         <f aca="false">IF($B68=0,"n/a",F26/$B68)</f>
@@ -9289,7 +9289,7 @@
       </c>
       <c r="C69" s="42" t="n">
         <f aca="false">C27/$B69</f>
-        <v>1.77845385964912</v>
+        <v>3.50203122807018</v>
       </c>
       <c r="D69" s="42" t="n">
         <f aca="false">D27/$B69</f>
@@ -9297,7 +9297,7 @@
       </c>
       <c r="E69" s="42" t="n">
         <f aca="false">E27/$B69</f>
-        <v>13.6820771929825</v>
+        <v>10.2539238596491</v>
       </c>
       <c r="F69" s="42" t="n">
         <f aca="false">F27/$B69</f>

</xml_diff>